<commit_message>
Fix CT27: confidentialityCode assente (non typeId) + riesecuzione completa
- CT27 (ID 468): corretto test case - rimuove confidentialityCode come da
  specifica CDA2_RSA_KO.xlsx (prima rimuoveva typeId causando HTTP 500
  senza workflowInstanceId, ora correttamente HTTP 400)
- Tutti 23 test con traceId e workflowInstanceId validi
- Colonna I (workflowInstanceId) ora presente per ID 468
</commit_message>
<xml_diff>
--- a/GATEWAY/A1_111_DLABSRLXX/D.Lab_Srl/OsteoEasy/2.0/report-checklist.xlsx
+++ b/GATEWAY/A1_111_DLABSRLXX/D.Lab_Srl/OsteoEasy/2.0/report-checklist.xlsx
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="690">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="691">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -390,13 +390,13 @@
     <t>VALIDAZIONE_TOKEN_JWT_RSA_KO</t>
   </si>
   <si>
-    <t>03/04/2026</t>
-  </si>
-  <si>
-    <t>2026-04-03T08:55:57+02:00</t>
-  </si>
-  <si>
-    <t>e4cbe928d3367379bb29becc62b6a271</t>
+    <t>05/04/2026</t>
+  </si>
+  <si>
+    <t>2026-04-05T08:46:57+02:00</t>
+  </si>
+  <si>
+    <t>88bf7c33f18868fce0485eca4876ab6b</t>
   </si>
   <si>
     <t>SI</t>
@@ -495,7 +495,7 @@
     <t>VALIDAZIONE_TOKEN_JWT_CAMPO_RSA_KO</t>
   </si>
   <si>
-    <t>16dbcf2db05f5d236691d07bf272b2c6</t>
+    <t>b201314daf4f83715601977b9e69502e</t>
   </si>
   <si>
     <t>VALIDAZIONE_TOKEN_JWT_CAMPO_CERT_VAC_KO</t>
@@ -1115,13 +1115,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 6" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>2026-04-03T08:55:58+02:00</t>
-  </si>
-  <si>
-    <t>f3e8211741752326f40bcc70611a5d7d</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.eab7ea2a56^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>7f517833e20770b07a3f0623e6a39885</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.5f015d0e0a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>Si e' verificato un errore durante l'operazione. Errore di validazione del documento CDA. Verificare il contenuto del documento e riprovare.</t>
@@ -1137,10 +1134,13 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 8" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>6290482be6ab3944900a533193ed8abf</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.771763e932^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>2026-04-05T08:46:58+02:00</t>
+  </si>
+  <si>
+    <t>1092d6abceb0441de8cfbfe88facd2c6</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.b20cca2eb1^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_RSA_CT9_KO</t>
@@ -1150,10 +1150,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 9" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>8925a9a26e0f147bde4d645f633ddead</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.3bb4251d43^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>054985100ddf44df6df9f1c9d6c16e93</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.af0eb4c6b2^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_RSA_CT10_KO</t>
@@ -1163,10 +1163,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 10" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>f957e6203e3bc87af35179f4b13dc90e</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.bbb899b1de^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>96875f4f4e866afee3915727f90c7a42</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.ab86552b27^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_RSA_CT13_KO</t>
@@ -1176,13 +1176,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 13" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>2026-04-03T08:55:59+02:00</t>
-  </si>
-  <si>
-    <t>0771b01e0f1fb116377ee9fabd753bbe</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.186999bd77^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>60096d146e015f489b2771c5103dfe09</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.bdf0e8f941^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_RSA_CT14_KO</t>
@@ -1192,10 +1189,13 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 14" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>a963b22cd7cde9192710f6d264da436d</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.f952ed1f3c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>2026-04-05T08:46:59+02:00</t>
+  </si>
+  <si>
+    <t>328e36daff3472dac4eb0fe56fe0b0df</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.df6b701edb^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_RSA_CT15_KO</t>
@@ -1205,10 +1205,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 15" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>c356c36d9fbab67b3c3dd59843b44948</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.708f92b7c0^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>b62f01005e616f4b1fc5d976b2f962c8</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.d463904d1a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_RSA_CT16_KO</t>
@@ -1218,13 +1218,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 16" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>2026-04-03T08:56:00+02:00</t>
-  </si>
-  <si>
-    <t>0fe3f7b3e99b578acb7586a39b845750</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.8127a1416d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>d5282b07adbbafdc30fde7940853c973</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.7c9f07619c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_RSA_CT17_KO</t>
@@ -1234,10 +1231,13 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 17" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>84297aec955c9eeb4c911ae6ee49f45c</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.8517eaadda^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>2026-04-05T08:47:00+02:00</t>
+  </si>
+  <si>
+    <t>868e33bbc9f116edc69dbbfd497083cd</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.837218d61b^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_RSA_CT18_KO</t>
@@ -1247,10 +1247,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 18" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>e7c274eb375320ce00e905f6fd2e1179</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.947422b0bd^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>1616926f49ab3696b95a50934a660430</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.9e36de85a4^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_RSA_CT19_KO</t>
@@ -1260,10 +1260,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 19" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>26c5d1b3e06dd6238ab65cc62efa212a</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.3f1f3284c9^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>b5207f1e554cabf7de71323e5ab1bcf8</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.4892c59b6b^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_RSA_CT20_KO</t>
@@ -1273,13 +1273,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 20" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>2026-04-03T08:56:01+02:00</t>
-  </si>
-  <si>
-    <t>4c1d170ce7f35b229c164970faa70921</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.641ed129c1^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>2eaa80c05d5d3583830b7fbec632313a</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.16906e0b9f^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_RSA_CT21_KO</t>
@@ -1289,10 +1286,13 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 21" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>dd1dab393f5514349139f284b880a281</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.98cae7d745^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>2026-04-05T08:47:01+02:00</t>
+  </si>
+  <si>
+    <t>772e6ec254edf91b76be07fabf085a91</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.10a40ffacb^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_RSA_CT22_KO</t>
@@ -1302,10 +1302,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 22" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>b4f2807e75d2cdd87b1ddb9b99ac29cd</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.8dca82b5dc^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>f607471fa5e4c99f38f1156d168aedb7</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.38f4f074e5^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_RSA_CT23_KO</t>
@@ -1315,13 +1315,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 23" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>2026-04-03T08:56:02+02:00</t>
-  </si>
-  <si>
-    <t>4b4225c36393a2fde7ed1636fcd97d9d</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.4bb3c6cbab^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>4ca491aa09dd165273331f33e20ad8da</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.219f921d1e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_PSS_CT6_KO</t>
@@ -1561,10 +1558,13 @@
 Il Documento CDA2 Referto Specialistica Ambulatoriale dovrà essere composto in modo da risultare valido dal punto di vista sintattico, semantico, terminologico. I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso dalla sezione "CASO DI TEST 24" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_OK" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>9fc297b462711c6a0c93e0c394ac55bf</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.559394b32c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>2026-04-05T08:46:56+02:00</t>
+  </si>
+  <si>
+    <t>69b5b697682013d3b62cde00d9e8959f</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.a02c4ac001^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_RSA_CT25</t>
@@ -1574,10 +1574,10 @@
 Il Documento CDA2 Referto Specialistica Ambulatoriale dovrà essere composto in modo da risultare valido dal punto di vista sintattico, semantico, terminologico. I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso dalla sezione "CASO DI TEST 25" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_OK" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>1c975a5d8d21a09f2fd72b0a1b1d84fd</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.12aad0cbef^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>c2772f9e9f4da061f179b08bd388ff91</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.009703c8bf^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_LDO_CT17</t>
@@ -1658,10 +1658,13 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 26" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>b418b517cbc0940ea77bd83e0012149b</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.29b5acc539^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>2026-04-05T08:47:02+02:00</t>
+  </si>
+  <si>
+    <t>ea53d60d79fd31be747333095e72cd49</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.7265ee8044^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_RAD_CT24_KO</t>
@@ -1713,7 +1716,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 27" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>af819f8409c307f6c87a1bcbf6fe25d3</t>
+    <t>c6449c069a5d36a97530b4264d9c9422</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.1908eae4de^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_PSS_CT22_KO</t>
@@ -1765,13 +1771,10 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 28" riportata nei documenti "casi di test RSA" e "CDA2_Referto_Specialistica_Ambulatoriale_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>2026-04-03T08:56:03+02:00</t>
-  </si>
-  <si>
-    <t>b1d4cdb3427cb7d71bd542bc5c93ee3c</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.6a844f08ee^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>0e83a642087369c79f47656fc09eea32</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.ab07c1eda2^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t>VALIDAZIONE_CDA2_PSS_CT23</t>
@@ -9375,13 +9378,13 @@
         <v>67</v>
       </c>
       <c r="G116" s="31" t="s">
+        <v>68</v>
+      </c>
+      <c r="H116" s="31" t="s">
         <v>264</v>
       </c>
-      <c r="H116" s="31" t="s">
+      <c r="I116" s="36" t="s">
         <v>265</v>
-      </c>
-      <c r="I116" s="36" t="s">
-        <v>266</v>
       </c>
       <c r="J116" s="32" t="s">
         <v>70</v>
@@ -9395,7 +9398,7 @@
         <v>70</v>
       </c>
       <c r="O116" s="32" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="P116" s="32" t="s">
         <v>53</v>
@@ -9407,7 +9410,7 @@
         <v>70</v>
       </c>
       <c r="S116" s="32" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T116" s="32"/>
       <c r="U116" s="33"/>
@@ -9427,16 +9430,16 @@
         <v>65</v>
       </c>
       <c r="D117" s="29" t="s">
+        <v>268</v>
+      </c>
+      <c r="E117" s="37" t="s">
         <v>269</v>
-      </c>
-      <c r="E117" s="37" t="s">
-        <v>270</v>
       </c>
       <c r="F117" s="31" t="s">
         <v>67</v>
       </c>
       <c r="G117" s="31" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="H117" s="31" t="s">
         <v>271</v>
@@ -9456,7 +9459,7 @@
         <v>70</v>
       </c>
       <c r="O117" s="32" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="P117" s="32" t="s">
         <v>53</v>
@@ -9468,7 +9471,7 @@
         <v>70</v>
       </c>
       <c r="S117" s="32" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T117" s="32"/>
       <c r="U117" s="33"/>
@@ -9497,7 +9500,7 @@
         <v>67</v>
       </c>
       <c r="G118" s="31" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="H118" s="31" t="s">
         <v>275</v>
@@ -9517,7 +9520,7 @@
         <v>70</v>
       </c>
       <c r="O118" s="32" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="P118" s="32" t="s">
         <v>53</v>
@@ -9529,7 +9532,7 @@
         <v>70</v>
       </c>
       <c r="S118" s="32" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T118" s="32"/>
       <c r="U118" s="33"/>
@@ -9558,7 +9561,7 @@
         <v>67</v>
       </c>
       <c r="G119" s="31" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="H119" s="31" t="s">
         <v>279</v>
@@ -9578,7 +9581,7 @@
         <v>70</v>
       </c>
       <c r="O119" s="32" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="P119" s="32" t="s">
         <v>53</v>
@@ -9590,7 +9593,7 @@
         <v>70</v>
       </c>
       <c r="S119" s="32" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T119" s="32"/>
       <c r="U119" s="33"/>
@@ -9619,13 +9622,13 @@
         <v>67</v>
       </c>
       <c r="G120" s="31" t="s">
+        <v>270</v>
+      </c>
+      <c r="H120" s="31" t="s">
         <v>283</v>
       </c>
-      <c r="H120" s="31" t="s">
+      <c r="I120" s="36" t="s">
         <v>284</v>
-      </c>
-      <c r="I120" s="36" t="s">
-        <v>285</v>
       </c>
       <c r="J120" s="32" t="s">
         <v>70</v>
@@ -9639,7 +9642,7 @@
         <v>70</v>
       </c>
       <c r="O120" s="32" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="P120" s="32" t="s">
         <v>53</v>
@@ -9651,7 +9654,7 @@
         <v>70</v>
       </c>
       <c r="S120" s="32" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T120" s="32"/>
       <c r="U120" s="33"/>
@@ -9671,16 +9674,16 @@
         <v>65</v>
       </c>
       <c r="D121" s="29" t="s">
+        <v>285</v>
+      </c>
+      <c r="E121" s="37" t="s">
         <v>286</v>
-      </c>
-      <c r="E121" s="37" t="s">
-        <v>287</v>
       </c>
       <c r="F121" s="31" t="s">
         <v>67</v>
       </c>
       <c r="G121" s="31" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="H121" s="31" t="s">
         <v>288</v>
@@ -9700,7 +9703,7 @@
         <v>70</v>
       </c>
       <c r="O121" s="32" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="P121" s="32" t="s">
         <v>53</v>
@@ -9712,7 +9715,7 @@
         <v>70</v>
       </c>
       <c r="S121" s="32" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T121" s="32"/>
       <c r="U121" s="33"/>
@@ -9741,7 +9744,7 @@
         <v>67</v>
       </c>
       <c r="G122" s="31" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="H122" s="31" t="s">
         <v>292</v>
@@ -9761,7 +9764,7 @@
         <v>70</v>
       </c>
       <c r="O122" s="32" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="P122" s="32" t="s">
         <v>53</v>
@@ -9773,7 +9776,7 @@
         <v>70</v>
       </c>
       <c r="S122" s="32" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T122" s="32"/>
       <c r="U122" s="33"/>
@@ -9802,13 +9805,13 @@
         <v>67</v>
       </c>
       <c r="G123" s="31" t="s">
+        <v>287</v>
+      </c>
+      <c r="H123" s="31" t="s">
         <v>296</v>
       </c>
-      <c r="H123" s="31" t="s">
+      <c r="I123" s="36" t="s">
         <v>297</v>
-      </c>
-      <c r="I123" s="36" t="s">
-        <v>298</v>
       </c>
       <c r="J123" s="32" t="s">
         <v>70</v>
@@ -9822,7 +9825,7 @@
         <v>70</v>
       </c>
       <c r="O123" s="32" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="P123" s="32" t="s">
         <v>53</v>
@@ -9834,7 +9837,7 @@
         <v>70</v>
       </c>
       <c r="S123" s="32" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T123" s="32"/>
       <c r="U123" s="33"/>
@@ -9854,16 +9857,16 @@
         <v>65</v>
       </c>
       <c r="D124" s="29" t="s">
+        <v>298</v>
+      </c>
+      <c r="E124" s="37" t="s">
         <v>299</v>
-      </c>
-      <c r="E124" s="37" t="s">
-        <v>300</v>
       </c>
       <c r="F124" s="31" t="s">
         <v>67</v>
       </c>
       <c r="G124" s="31" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="H124" s="31" t="s">
         <v>301</v>
@@ -9883,7 +9886,7 @@
         <v>70</v>
       </c>
       <c r="O124" s="32" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="P124" s="32" t="s">
         <v>53</v>
@@ -9895,7 +9898,7 @@
         <v>70</v>
       </c>
       <c r="S124" s="32" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T124" s="32"/>
       <c r="U124" s="33"/>
@@ -9924,7 +9927,7 @@
         <v>67</v>
       </c>
       <c r="G125" s="31" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="H125" s="31" t="s">
         <v>305</v>
@@ -9944,7 +9947,7 @@
         <v>70</v>
       </c>
       <c r="O125" s="32" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="P125" s="32" t="s">
         <v>53</v>
@@ -9956,7 +9959,7 @@
         <v>70</v>
       </c>
       <c r="S125" s="32" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T125" s="32"/>
       <c r="U125" s="33"/>
@@ -9985,7 +9988,7 @@
         <v>67</v>
       </c>
       <c r="G126" s="31" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="H126" s="31" t="s">
         <v>309</v>
@@ -10005,7 +10008,7 @@
         <v>70</v>
       </c>
       <c r="O126" s="32" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="P126" s="32" t="s">
         <v>53</v>
@@ -10017,7 +10020,7 @@
         <v>70</v>
       </c>
       <c r="S126" s="32" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T126" s="32"/>
       <c r="U126" s="33"/>
@@ -10046,13 +10049,13 @@
         <v>67</v>
       </c>
       <c r="G127" s="31" t="s">
+        <v>300</v>
+      </c>
+      <c r="H127" s="31" t="s">
         <v>313</v>
       </c>
-      <c r="H127" s="31" t="s">
+      <c r="I127" s="36" t="s">
         <v>314</v>
-      </c>
-      <c r="I127" s="36" t="s">
-        <v>315</v>
       </c>
       <c r="J127" s="32" t="s">
         <v>70</v>
@@ -10066,7 +10069,7 @@
         <v>70</v>
       </c>
       <c r="O127" s="32" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="P127" s="32" t="s">
         <v>53</v>
@@ -10078,7 +10081,7 @@
         <v>70</v>
       </c>
       <c r="S127" s="32" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T127" s="32"/>
       <c r="U127" s="33"/>
@@ -10098,16 +10101,16 @@
         <v>65</v>
       </c>
       <c r="D128" s="29" t="s">
+        <v>315</v>
+      </c>
+      <c r="E128" s="37" t="s">
         <v>316</v>
-      </c>
-      <c r="E128" s="37" t="s">
-        <v>317</v>
       </c>
       <c r="F128" s="31" t="s">
         <v>67</v>
       </c>
       <c r="G128" s="31" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="H128" s="31" t="s">
         <v>318</v>
@@ -10127,7 +10130,7 @@
         <v>70</v>
       </c>
       <c r="O128" s="32" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="P128" s="32" t="s">
         <v>53</v>
@@ -10139,7 +10142,7 @@
         <v>70</v>
       </c>
       <c r="S128" s="32" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T128" s="32"/>
       <c r="U128" s="33"/>
@@ -10168,7 +10171,7 @@
         <v>67</v>
       </c>
       <c r="G129" s="31" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="H129" s="31" t="s">
         <v>322</v>
@@ -10188,7 +10191,7 @@
         <v>70</v>
       </c>
       <c r="O129" s="32" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="P129" s="32" t="s">
         <v>53</v>
@@ -10200,7 +10203,7 @@
         <v>70</v>
       </c>
       <c r="S129" s="32" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T129" s="32"/>
       <c r="U129" s="33"/>
@@ -10229,13 +10232,13 @@
         <v>67</v>
       </c>
       <c r="G130" s="31" t="s">
+        <v>317</v>
+      </c>
+      <c r="H130" s="31" t="s">
         <v>326</v>
       </c>
-      <c r="H130" s="31" t="s">
+      <c r="I130" s="36" t="s">
         <v>327</v>
-      </c>
-      <c r="I130" s="36" t="s">
-        <v>328</v>
       </c>
       <c r="J130" s="32" t="s">
         <v>70</v>
@@ -10249,7 +10252,7 @@
         <v>70</v>
       </c>
       <c r="O130" s="32" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="P130" s="32" t="s">
         <v>53</v>
@@ -10261,7 +10264,7 @@
         <v>70</v>
       </c>
       <c r="S130" s="32" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T130" s="32"/>
       <c r="U130" s="33"/>
@@ -10281,10 +10284,10 @@
         <v>61</v>
       </c>
       <c r="D131" s="29" t="s">
+        <v>328</v>
+      </c>
+      <c r="E131" s="37" t="s">
         <v>329</v>
-      </c>
-      <c r="E131" s="37" t="s">
-        <v>330</v>
       </c>
       <c r="F131" s="31"/>
       <c r="G131" s="31"/>
@@ -10322,10 +10325,10 @@
         <v>61</v>
       </c>
       <c r="D132" s="29" t="s">
+        <v>330</v>
+      </c>
+      <c r="E132" s="37" t="s">
         <v>331</v>
-      </c>
-      <c r="E132" s="37" t="s">
-        <v>332</v>
       </c>
       <c r="F132" s="31"/>
       <c r="G132" s="31"/>
@@ -10363,10 +10366,10 @@
         <v>61</v>
       </c>
       <c r="D133" s="29" t="s">
+        <v>332</v>
+      </c>
+      <c r="E133" s="37" t="s">
         <v>333</v>
-      </c>
-      <c r="E133" s="37" t="s">
-        <v>334</v>
       </c>
       <c r="F133" s="31"/>
       <c r="G133" s="31"/>
@@ -10404,10 +10407,10 @@
         <v>61</v>
       </c>
       <c r="D134" s="29" t="s">
+        <v>334</v>
+      </c>
+      <c r="E134" s="37" t="s">
         <v>335</v>
-      </c>
-      <c r="E134" s="37" t="s">
-        <v>336</v>
       </c>
       <c r="F134" s="31"/>
       <c r="G134" s="31"/>
@@ -10445,10 +10448,10 @@
         <v>61</v>
       </c>
       <c r="D135" s="29" t="s">
+        <v>336</v>
+      </c>
+      <c r="E135" s="37" t="s">
         <v>337</v>
-      </c>
-      <c r="E135" s="37" t="s">
-        <v>338</v>
       </c>
       <c r="F135" s="31"/>
       <c r="G135" s="31"/>
@@ -10486,10 +10489,10 @@
         <v>61</v>
       </c>
       <c r="D136" s="29" t="s">
+        <v>338</v>
+      </c>
+      <c r="E136" s="37" t="s">
         <v>339</v>
-      </c>
-      <c r="E136" s="37" t="s">
-        <v>340</v>
       </c>
       <c r="F136" s="31"/>
       <c r="G136" s="31"/>
@@ -10527,10 +10530,10 @@
         <v>61</v>
       </c>
       <c r="D137" s="29" t="s">
+        <v>340</v>
+      </c>
+      <c r="E137" s="37" t="s">
         <v>341</v>
-      </c>
-      <c r="E137" s="37" t="s">
-        <v>342</v>
       </c>
       <c r="F137" s="31"/>
       <c r="G137" s="31"/>
@@ -10568,10 +10571,10 @@
         <v>61</v>
       </c>
       <c r="D138" s="29" t="s">
+        <v>342</v>
+      </c>
+      <c r="E138" s="37" t="s">
         <v>343</v>
-      </c>
-      <c r="E138" s="37" t="s">
-        <v>344</v>
       </c>
       <c r="F138" s="31"/>
       <c r="G138" s="31"/>
@@ -10609,10 +10612,10 @@
         <v>61</v>
       </c>
       <c r="D139" s="29" t="s">
+        <v>344</v>
+      </c>
+      <c r="E139" s="37" t="s">
         <v>345</v>
-      </c>
-      <c r="E139" s="37" t="s">
-        <v>346</v>
       </c>
       <c r="F139" s="31"/>
       <c r="G139" s="31"/>
@@ -10650,10 +10653,10 @@
         <v>61</v>
       </c>
       <c r="D140" s="29" t="s">
+        <v>346</v>
+      </c>
+      <c r="E140" s="37" t="s">
         <v>347</v>
-      </c>
-      <c r="E140" s="37" t="s">
-        <v>348</v>
       </c>
       <c r="F140" s="31"/>
       <c r="G140" s="31"/>
@@ -10691,10 +10694,10 @@
         <v>61</v>
       </c>
       <c r="D141" s="29" t="s">
+        <v>348</v>
+      </c>
+      <c r="E141" s="37" t="s">
         <v>349</v>
-      </c>
-      <c r="E141" s="37" t="s">
-        <v>350</v>
       </c>
       <c r="F141" s="31"/>
       <c r="G141" s="31"/>
@@ -10732,10 +10735,10 @@
         <v>61</v>
       </c>
       <c r="D142" s="29" t="s">
+        <v>350</v>
+      </c>
+      <c r="E142" s="37" t="s">
         <v>351</v>
-      </c>
-      <c r="E142" s="37" t="s">
-        <v>352</v>
       </c>
       <c r="F142" s="31"/>
       <c r="G142" s="31"/>
@@ -10773,10 +10776,10 @@
         <v>61</v>
       </c>
       <c r="D143" s="29" t="s">
+        <v>352</v>
+      </c>
+      <c r="E143" s="37" t="s">
         <v>353</v>
-      </c>
-      <c r="E143" s="37" t="s">
-        <v>354</v>
       </c>
       <c r="F143" s="31"/>
       <c r="G143" s="31"/>
@@ -10814,10 +10817,10 @@
         <v>61</v>
       </c>
       <c r="D144" s="29" t="s">
+        <v>354</v>
+      </c>
+      <c r="E144" s="37" t="s">
         <v>355</v>
-      </c>
-      <c r="E144" s="37" t="s">
-        <v>356</v>
       </c>
       <c r="F144" s="31"/>
       <c r="G144" s="31"/>
@@ -10855,10 +10858,10 @@
         <v>61</v>
       </c>
       <c r="D145" s="29" t="s">
+        <v>356</v>
+      </c>
+      <c r="E145" s="37" t="s">
         <v>357</v>
-      </c>
-      <c r="E145" s="37" t="s">
-        <v>358</v>
       </c>
       <c r="F145" s="31"/>
       <c r="G145" s="31"/>
@@ -10896,10 +10899,10 @@
         <v>50</v>
       </c>
       <c r="D146" s="29" t="s">
+        <v>358</v>
+      </c>
+      <c r="E146" s="37" t="s">
         <v>359</v>
-      </c>
-      <c r="E146" s="37" t="s">
-        <v>360</v>
       </c>
       <c r="F146" s="31"/>
       <c r="G146" s="31"/>
@@ -10937,10 +10940,10 @@
         <v>50</v>
       </c>
       <c r="D147" s="29" t="s">
+        <v>360</v>
+      </c>
+      <c r="E147" s="37" t="s">
         <v>361</v>
-      </c>
-      <c r="E147" s="37" t="s">
-        <v>362</v>
       </c>
       <c r="F147" s="31"/>
       <c r="G147" s="31"/>
@@ -10975,13 +10978,13 @@
         <v>49</v>
       </c>
       <c r="C148" s="35" t="s">
+        <v>362</v>
+      </c>
+      <c r="D148" s="29" t="s">
         <v>363</v>
       </c>
-      <c r="D148" s="29" t="s">
+      <c r="E148" s="37" t="s">
         <v>364</v>
-      </c>
-      <c r="E148" s="37" t="s">
-        <v>365</v>
       </c>
       <c r="F148" s="31"/>
       <c r="G148" s="31"/>
@@ -11016,13 +11019,13 @@
         <v>49</v>
       </c>
       <c r="C149" s="35" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D149" s="29" t="s">
+        <v>365</v>
+      </c>
+      <c r="E149" s="37" t="s">
         <v>366</v>
-      </c>
-      <c r="E149" s="37" t="s">
-        <v>367</v>
       </c>
       <c r="F149" s="31"/>
       <c r="G149" s="31"/>
@@ -11057,13 +11060,13 @@
         <v>49</v>
       </c>
       <c r="C150" s="35" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D150" s="29" t="s">
+        <v>367</v>
+      </c>
+      <c r="E150" s="37" t="s">
         <v>368</v>
-      </c>
-      <c r="E150" s="37" t="s">
-        <v>369</v>
       </c>
       <c r="F150" s="31"/>
       <c r="G150" s="31"/>
@@ -11098,10 +11101,10 @@
         <v>49</v>
       </c>
       <c r="C151" s="35" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D151" s="29" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E151" s="37" t="s">
         <v>57</v>
@@ -11139,10 +11142,10 @@
         <v>49</v>
       </c>
       <c r="C152" s="35" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D152" s="29" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="E152" s="37" t="s">
         <v>80</v>
@@ -11180,13 +11183,13 @@
         <v>49</v>
       </c>
       <c r="C153" s="35" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D153" s="29" t="s">
+        <v>371</v>
+      </c>
+      <c r="E153" s="37" t="s">
         <v>372</v>
-      </c>
-      <c r="E153" s="37" t="s">
-        <v>373</v>
       </c>
       <c r="F153" s="31"/>
       <c r="G153" s="31"/>
@@ -11223,13 +11226,13 @@
         <v>49</v>
       </c>
       <c r="C154" s="35" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D154" s="29" t="s">
+        <v>373</v>
+      </c>
+      <c r="E154" s="37" t="s">
         <v>374</v>
-      </c>
-      <c r="E154" s="37" t="s">
-        <v>375</v>
       </c>
       <c r="F154" s="31"/>
       <c r="G154" s="31"/>
@@ -11264,13 +11267,13 @@
         <v>49</v>
       </c>
       <c r="C155" s="35" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D155" s="29" t="s">
+        <v>375</v>
+      </c>
+      <c r="E155" s="37" t="s">
         <v>376</v>
-      </c>
-      <c r="E155" s="37" t="s">
-        <v>377</v>
       </c>
       <c r="F155" s="31"/>
       <c r="G155" s="31"/>
@@ -11305,13 +11308,13 @@
         <v>49</v>
       </c>
       <c r="C156" s="35" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D156" s="29" t="s">
+        <v>377</v>
+      </c>
+      <c r="E156" s="37" t="s">
         <v>378</v>
-      </c>
-      <c r="E156" s="37" t="s">
-        <v>379</v>
       </c>
       <c r="F156" s="31"/>
       <c r="G156" s="31"/>
@@ -11346,13 +11349,13 @@
         <v>49</v>
       </c>
       <c r="C157" s="35" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D157" s="29" t="s">
+        <v>379</v>
+      </c>
+      <c r="E157" s="37" t="s">
         <v>380</v>
-      </c>
-      <c r="E157" s="37" t="s">
-        <v>381</v>
       </c>
       <c r="F157" s="31"/>
       <c r="G157" s="31"/>
@@ -11387,13 +11390,13 @@
         <v>49</v>
       </c>
       <c r="C158" s="35" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D158" s="29" t="s">
+        <v>381</v>
+      </c>
+      <c r="E158" s="37" t="s">
         <v>382</v>
-      </c>
-      <c r="E158" s="37" t="s">
-        <v>383</v>
       </c>
       <c r="F158" s="31"/>
       <c r="G158" s="31"/>
@@ -11428,13 +11431,13 @@
         <v>49</v>
       </c>
       <c r="C159" s="35" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D159" s="29" t="s">
+        <v>383</v>
+      </c>
+      <c r="E159" s="37" t="s">
         <v>384</v>
-      </c>
-      <c r="E159" s="37" t="s">
-        <v>385</v>
       </c>
       <c r="F159" s="31"/>
       <c r="G159" s="31"/>
@@ -11469,13 +11472,13 @@
         <v>49</v>
       </c>
       <c r="C160" s="35" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D160" s="29" t="s">
+        <v>385</v>
+      </c>
+      <c r="E160" s="37" t="s">
         <v>386</v>
-      </c>
-      <c r="E160" s="37" t="s">
-        <v>387</v>
       </c>
       <c r="F160" s="31"/>
       <c r="G160" s="31"/>
@@ -11510,13 +11513,13 @@
         <v>49</v>
       </c>
       <c r="C161" s="35" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D161" s="29" t="s">
+        <v>387</v>
+      </c>
+      <c r="E161" s="37" t="s">
         <v>388</v>
-      </c>
-      <c r="E161" s="37" t="s">
-        <v>389</v>
       </c>
       <c r="F161" s="31"/>
       <c r="G161" s="31"/>
@@ -11551,13 +11554,13 @@
         <v>49</v>
       </c>
       <c r="C162" s="35" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D162" s="29" t="s">
+        <v>389</v>
+      </c>
+      <c r="E162" s="37" t="s">
         <v>390</v>
-      </c>
-      <c r="E162" s="37" t="s">
-        <v>391</v>
       </c>
       <c r="F162" s="31"/>
       <c r="G162" s="31"/>
@@ -11592,13 +11595,13 @@
         <v>49</v>
       </c>
       <c r="C163" s="35" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D163" s="29" t="s">
+        <v>391</v>
+      </c>
+      <c r="E163" s="37" t="s">
         <v>392</v>
-      </c>
-      <c r="E163" s="37" t="s">
-        <v>393</v>
       </c>
       <c r="F163" s="31"/>
       <c r="G163" s="31"/>
@@ -11636,16 +11639,16 @@
         <v>65</v>
       </c>
       <c r="D164" s="29" t="s">
+        <v>393</v>
+      </c>
+      <c r="E164" s="37" t="s">
         <v>394</v>
-      </c>
-      <c r="E164" s="37" t="s">
-        <v>395</v>
       </c>
       <c r="F164" s="31" t="s">
         <v>67</v>
       </c>
       <c r="G164" s="31" t="s">
-        <v>68</v>
+        <v>395</v>
       </c>
       <c r="H164" s="31" t="s">
         <v>396</v>
@@ -12096,7 +12099,7 @@
         <v>49</v>
       </c>
       <c r="C175" s="35" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D175" s="29" t="s">
         <v>420</v>
@@ -12149,13 +12152,13 @@
         <v>67</v>
       </c>
       <c r="G176" s="29" t="s">
-        <v>326</v>
+        <v>424</v>
       </c>
       <c r="H176" s="29" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="I176" s="29" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="J176" s="32" t="s">
         <v>70</v>
@@ -12169,7 +12172,7 @@
         <v>70</v>
       </c>
       <c r="O176" s="29" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="P176" s="32" t="s">
         <v>53</v>
@@ -12181,7 +12184,7 @@
         <v>70</v>
       </c>
       <c r="S176" s="29" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T176" s="32"/>
       <c r="U176" s="29"/>
@@ -12201,10 +12204,10 @@
         <v>63</v>
       </c>
       <c r="D177" s="29" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="E177" s="37" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="F177" s="29"/>
       <c r="G177" s="29"/>
@@ -12242,10 +12245,10 @@
         <v>77</v>
       </c>
       <c r="D178" s="29" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="E178" s="37" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="F178" s="29"/>
       <c r="G178" s="29"/>
@@ -12283,10 +12286,10 @@
         <v>73</v>
       </c>
       <c r="D179" s="29" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E179" s="37" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="F179" s="29"/>
       <c r="G179" s="29"/>
@@ -12324,10 +12327,10 @@
         <v>75</v>
       </c>
       <c r="D180" s="29" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="E180" s="37" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="F180" s="29"/>
       <c r="G180" s="29"/>
@@ -12365,10 +12368,10 @@
         <v>50</v>
       </c>
       <c r="D181" s="29" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E181" s="37" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F181" s="29"/>
       <c r="G181" s="29"/>
@@ -12406,10 +12409,10 @@
         <v>59</v>
       </c>
       <c r="D182" s="29" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="E182" s="37" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="F182" s="29"/>
       <c r="G182" s="29"/>
@@ -12447,21 +12450,23 @@
         <v>65</v>
       </c>
       <c r="D183" s="29" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="E183" s="37" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F183" s="29" t="s">
         <v>67</v>
       </c>
       <c r="G183" s="29" t="s">
-        <v>326</v>
+        <v>424</v>
       </c>
       <c r="H183" s="29" t="s">
-        <v>440</v>
-      </c>
-      <c r="I183" s="29"/>
+        <v>441</v>
+      </c>
+      <c r="I183" s="29" t="s">
+        <v>442</v>
+      </c>
       <c r="J183" s="32" t="s">
         <v>70</v>
       </c>
@@ -12474,7 +12479,7 @@
         <v>70</v>
       </c>
       <c r="O183" s="29" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="P183" s="32" t="s">
         <v>53</v>
@@ -12486,7 +12491,7 @@
         <v>70</v>
       </c>
       <c r="S183" s="29" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T183" s="32"/>
       <c r="U183" s="29"/>
@@ -12506,10 +12511,10 @@
         <v>61</v>
       </c>
       <c r="D184" s="29" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="E184" s="37" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="F184" s="29"/>
       <c r="G184" s="29"/>
@@ -12544,13 +12549,13 @@
         <v>49</v>
       </c>
       <c r="C185" s="35" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D185" s="29" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="E185" s="37" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="F185" s="29"/>
       <c r="G185" s="29"/>
@@ -12588,10 +12593,10 @@
         <v>63</v>
       </c>
       <c r="D186" s="29" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="E186" s="37" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="F186" s="31"/>
       <c r="G186" s="31"/>
@@ -12629,10 +12634,10 @@
         <v>63</v>
       </c>
       <c r="D187" s="29" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="E187" s="37" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="F187" s="31"/>
       <c r="G187" s="31"/>
@@ -12670,10 +12675,10 @@
         <v>50</v>
       </c>
       <c r="D188" s="35" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="E188" s="37" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="F188" s="31"/>
       <c r="G188" s="31"/>
@@ -12711,10 +12716,10 @@
         <v>63</v>
       </c>
       <c r="D189" s="29" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="E189" s="37" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="F189" s="31"/>
       <c r="G189" s="31"/>
@@ -12752,22 +12757,22 @@
         <v>65</v>
       </c>
       <c r="D190" s="29" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="E190" s="37" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="F190" s="31" t="s">
         <v>67</v>
       </c>
       <c r="G190" s="31" t="s">
-        <v>455</v>
+        <v>424</v>
       </c>
       <c r="H190" s="31" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="I190" s="36" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="J190" s="32" t="s">
         <v>70</v>
@@ -12781,7 +12786,7 @@
         <v>70</v>
       </c>
       <c r="O190" s="32" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="P190" s="32" t="s">
         <v>53</v>
@@ -12793,7 +12798,7 @@
         <v>70</v>
       </c>
       <c r="S190" s="32" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="T190" s="32"/>
       <c r="U190" s="33"/>
@@ -12813,10 +12818,10 @@
         <v>61</v>
       </c>
       <c r="D191" s="29" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="E191" s="37" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="F191" s="31"/>
       <c r="G191" s="31"/>
@@ -12854,10 +12859,10 @@
         <v>61</v>
       </c>
       <c r="D192" s="29" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="E192" s="37" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F192" s="31"/>
       <c r="G192" s="31"/>
@@ -12895,10 +12900,10 @@
         <v>61</v>
       </c>
       <c r="D193" s="29" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="E193" s="40" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="F193" s="31"/>
       <c r="G193" s="31"/>
@@ -12933,13 +12938,13 @@
         <v>49</v>
       </c>
       <c r="C194" s="35" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D194" s="29" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="E194" s="40" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="F194" s="31"/>
       <c r="G194" s="31"/>
@@ -12974,13 +12979,13 @@
         <v>49</v>
       </c>
       <c r="C195" s="35" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D195" s="29" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="E195" s="40" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F195" s="31"/>
       <c r="G195" s="31"/>
@@ -13015,13 +13020,13 @@
         <v>49</v>
       </c>
       <c r="C196" s="35" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D196" s="29" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E196" s="40" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="F196" s="31"/>
       <c r="G196" s="31"/>
@@ -13056,13 +13061,13 @@
         <v>49</v>
       </c>
       <c r="C197" s="35" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D197" s="29" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E197" s="40" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="F197" s="31"/>
       <c r="G197" s="31"/>
@@ -13097,13 +13102,13 @@
         <v>49</v>
       </c>
       <c r="C198" s="35" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D198" s="29" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="E198" s="40" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="F198" s="31"/>
       <c r="G198" s="31"/>
@@ -13138,13 +13143,13 @@
         <v>49</v>
       </c>
       <c r="C199" s="35" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D199" s="29" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="E199" s="40" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="F199" s="31"/>
       <c r="G199" s="31"/>
@@ -13179,13 +13184,13 @@
         <v>49</v>
       </c>
       <c r="C200" s="35" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D200" s="29" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="E200" s="40" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="F200" s="31"/>
       <c r="G200" s="31"/>
@@ -13220,13 +13225,13 @@
         <v>49</v>
       </c>
       <c r="C201" s="35" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D201" s="29" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="E201" s="40" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F201" s="31"/>
       <c r="G201" s="31"/>
@@ -13261,13 +13266,13 @@
         <v>49</v>
       </c>
       <c r="C202" s="35" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D202" s="29" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="E202" s="40" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F202" s="31"/>
       <c r="G202" s="31"/>
@@ -13302,13 +13307,13 @@
         <v>49</v>
       </c>
       <c r="C203" s="35" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D203" s="29" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="E203" s="40" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="F203" s="31"/>
       <c r="G203" s="31"/>
@@ -13343,10 +13348,10 @@
         <v>49</v>
       </c>
       <c r="C204" s="35" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D204" s="29" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="E204" s="37" t="s">
         <v>80</v>
@@ -13384,10 +13389,10 @@
         <v>49</v>
       </c>
       <c r="C205" s="35" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D205" s="29" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="E205" s="37" t="s">
         <v>90</v>
@@ -13427,13 +13432,13 @@
         <v>49</v>
       </c>
       <c r="C206" s="35" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D206" s="29" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="E206" s="40" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="F206" s="31"/>
       <c r="G206" s="31"/>
@@ -13468,13 +13473,13 @@
         <v>49</v>
       </c>
       <c r="C207" s="35" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D207" s="29" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="E207" s="40" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="F207" s="31"/>
       <c r="G207" s="31"/>
@@ -13509,13 +13514,13 @@
         <v>49</v>
       </c>
       <c r="C208" s="35" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D208" s="29" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="E208" s="40" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F208" s="31"/>
       <c r="G208" s="31"/>
@@ -13550,13 +13555,13 @@
         <v>49</v>
       </c>
       <c r="C209" s="35" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D209" s="29" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="E209" s="40" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="F209" s="31"/>
       <c r="G209" s="31"/>
@@ -13591,13 +13596,13 @@
         <v>49</v>
       </c>
       <c r="C210" s="35" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D210" s="29" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="E210" s="40" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F210" s="31"/>
       <c r="G210" s="31"/>
@@ -13632,13 +13637,13 @@
         <v>49</v>
       </c>
       <c r="C211" s="35" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D211" s="29" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E211" s="40" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="F211" s="31"/>
       <c r="G211" s="31"/>
@@ -13673,13 +13678,13 @@
         <v>49</v>
       </c>
       <c r="C212" s="35" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D212" s="29" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="E212" s="40" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F212" s="31"/>
       <c r="G212" s="31"/>
@@ -13714,13 +13719,13 @@
         <v>49</v>
       </c>
       <c r="C213" s="35" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D213" s="29" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="E213" s="40" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="F213" s="31"/>
       <c r="G213" s="31"/>
@@ -13755,13 +13760,13 @@
         <v>49</v>
       </c>
       <c r="C214" s="35" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D214" s="29" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="E214" s="40" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="F214" s="31"/>
       <c r="G214" s="31"/>
@@ -13796,13 +13801,13 @@
         <v>49</v>
       </c>
       <c r="C215" s="35" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D215" s="29" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="E215" s="40" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F215" s="31"/>
       <c r="G215" s="31"/>
@@ -13837,13 +13842,13 @@
         <v>49</v>
       </c>
       <c r="C216" s="35" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D216" s="29" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E216" s="40" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="F216" s="31"/>
       <c r="G216" s="31"/>
@@ -13878,13 +13883,13 @@
         <v>49</v>
       </c>
       <c r="C217" s="35" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D217" s="29" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E217" s="40" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="F217" s="31"/>
       <c r="G217" s="31"/>
@@ -13919,13 +13924,13 @@
         <v>49</v>
       </c>
       <c r="C218" s="35" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D218" s="29" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="E218" s="40" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F218" s="31"/>
       <c r="G218" s="31"/>
@@ -13960,10 +13965,10 @@
         <v>49</v>
       </c>
       <c r="C219" s="35" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D219" s="29" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E219" s="37" t="s">
         <v>80</v>
@@ -14001,10 +14006,10 @@
         <v>49</v>
       </c>
       <c r="C220" s="35" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D220" s="29" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="E220" s="37" t="s">
         <v>90</v>
@@ -14044,13 +14049,13 @@
         <v>49</v>
       </c>
       <c r="C221" s="35" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D221" s="29" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="E221" s="40" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="F221" s="31"/>
       <c r="G221" s="31"/>
@@ -14085,13 +14090,13 @@
         <v>49</v>
       </c>
       <c r="C222" s="35" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D222" s="29" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="E222" s="40" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="F222" s="31"/>
       <c r="G222" s="31"/>
@@ -14126,13 +14131,13 @@
         <v>49</v>
       </c>
       <c r="C223" s="35" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D223" s="29" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="E223" s="40" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="F223" s="31"/>
       <c r="G223" s="31"/>
@@ -14167,13 +14172,13 @@
         <v>49</v>
       </c>
       <c r="C224" s="35" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D224" s="29" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="E224" s="40" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="F224" s="31"/>
       <c r="G224" s="31"/>
@@ -14208,13 +14213,13 @@
         <v>49</v>
       </c>
       <c r="C225" s="35" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D225" s="29" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="E225" s="40" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="F225" s="31"/>
       <c r="G225" s="31"/>
@@ -14249,13 +14254,13 @@
         <v>49</v>
       </c>
       <c r="C226" s="35" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D226" s="29" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="E226" s="40" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="F226" s="31"/>
       <c r="G226" s="31"/>
@@ -14290,13 +14295,13 @@
         <v>49</v>
       </c>
       <c r="C227" s="35" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D227" s="29" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="E227" s="40" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="F227" s="31"/>
       <c r="G227" s="31"/>
@@ -14331,13 +14336,13 @@
         <v>49</v>
       </c>
       <c r="C228" s="35" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D228" s="29" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="E228" s="40" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="F228" s="31"/>
       <c r="G228" s="31"/>
@@ -14372,13 +14377,13 @@
         <v>49</v>
       </c>
       <c r="C229" s="35" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D229" s="29" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="E229" s="40" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="F229" s="31"/>
       <c r="G229" s="31"/>
@@ -14413,13 +14418,13 @@
         <v>49</v>
       </c>
       <c r="C230" s="35" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D230" s="29" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="E230" s="40" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="F230" s="31"/>
       <c r="G230" s="31"/>
@@ -14454,13 +14459,13 @@
         <v>49</v>
       </c>
       <c r="C231" s="35" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D231" s="29" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="E231" s="40" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F231" s="31"/>
       <c r="G231" s="31"/>
@@ -14495,13 +14500,13 @@
         <v>49</v>
       </c>
       <c r="C232" s="35" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D232" s="29" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="E232" s="40" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F232" s="31"/>
       <c r="G232" s="31"/>
@@ -14536,13 +14541,13 @@
         <v>49</v>
       </c>
       <c r="C233" s="35" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D233" s="29" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="E233" s="40" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F233" s="31"/>
       <c r="G233" s="31"/>
@@ -14577,10 +14582,10 @@
         <v>49</v>
       </c>
       <c r="C234" s="35" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D234" s="29" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="E234" s="37" t="s">
         <v>80</v>
@@ -14618,10 +14623,10 @@
         <v>49</v>
       </c>
       <c r="C235" s="35" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="D235" s="29" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="E235" s="37" t="s">
         <v>90</v>
@@ -14661,13 +14666,13 @@
         <v>49</v>
       </c>
       <c r="C236" s="42" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D236" s="41" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="E236" s="40" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="F236" s="43"/>
       <c r="G236" s="43"/>
@@ -14702,13 +14707,13 @@
         <v>49</v>
       </c>
       <c r="C237" s="42" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D237" s="41" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="E237" s="40" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="F237" s="43"/>
       <c r="G237" s="43"/>
@@ -14743,13 +14748,13 @@
         <v>49</v>
       </c>
       <c r="C238" s="42" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D238" s="41" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="E238" s="40" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="F238" s="43"/>
       <c r="G238" s="43"/>
@@ -14784,13 +14789,13 @@
         <v>49</v>
       </c>
       <c r="C239" s="42" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D239" s="41" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="E239" s="40" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="F239" s="43"/>
       <c r="G239" s="43"/>
@@ -14825,13 +14830,13 @@
         <v>49</v>
       </c>
       <c r="C240" s="42" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D240" s="41" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="E240" s="40" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="F240" s="43"/>
       <c r="G240" s="43"/>
@@ -14866,13 +14871,13 @@
         <v>49</v>
       </c>
       <c r="C241" s="42" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D241" s="41" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="E241" s="40" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="F241" s="43"/>
       <c r="G241" s="43"/>
@@ -14907,13 +14912,13 @@
         <v>49</v>
       </c>
       <c r="C242" s="42" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D242" s="41" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="E242" s="40" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="F242" s="43"/>
       <c r="G242" s="43"/>
@@ -14948,13 +14953,13 @@
         <v>49</v>
       </c>
       <c r="C243" s="42" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D243" s="41" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="E243" s="40" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="F243" s="43"/>
       <c r="G243" s="43"/>
@@ -14989,10 +14994,10 @@
         <v>49</v>
       </c>
       <c r="C244" s="42" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D244" s="41" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="E244" s="40" t="s">
         <v>80</v>
@@ -15030,10 +15035,10 @@
         <v>49</v>
       </c>
       <c r="C245" s="42" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D245" s="41" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="E245" s="40" t="s">
         <v>90</v>
@@ -15073,13 +15078,13 @@
         <v>49</v>
       </c>
       <c r="C246" s="62" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D246" s="61" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="E246" s="63" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="F246" s="64"/>
       <c r="G246" s="64"/>
@@ -15114,13 +15119,13 @@
         <v>49</v>
       </c>
       <c r="C247" s="62" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D247" s="61" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="E247" s="63" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="F247" s="64"/>
       <c r="G247" s="64"/>
@@ -15155,13 +15160,13 @@
         <v>49</v>
       </c>
       <c r="C248" s="62" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D248" s="61" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="E248" s="63" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="F248" s="64"/>
       <c r="G248" s="64"/>
@@ -15196,13 +15201,13 @@
         <v>49</v>
       </c>
       <c r="C249" s="62" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D249" s="61" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="E249" s="63" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="F249" s="64"/>
       <c r="G249" s="64"/>
@@ -15237,13 +15242,13 @@
         <v>49</v>
       </c>
       <c r="C250" s="62" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D250" s="61" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="E250" s="63" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="F250" s="64"/>
       <c r="G250" s="64"/>
@@ -15278,13 +15283,13 @@
         <v>49</v>
       </c>
       <c r="C251" s="62" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D251" s="61" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="E251" s="63" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="F251" s="64"/>
       <c r="G251" s="64"/>
@@ -15319,13 +15324,13 @@
         <v>49</v>
       </c>
       <c r="C252" s="62" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D252" s="61" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="E252" s="63" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="F252" s="64"/>
       <c r="G252" s="64"/>
@@ -15360,13 +15365,13 @@
         <v>49</v>
       </c>
       <c r="C253" s="62" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D253" s="61" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="E253" s="63" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="F253" s="64"/>
       <c r="G253" s="64"/>
@@ -15401,13 +15406,13 @@
         <v>49</v>
       </c>
       <c r="C254" s="62" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D254" s="61" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="E254" s="63" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="F254" s="64"/>
       <c r="G254" s="64"/>
@@ -15442,13 +15447,13 @@
         <v>49</v>
       </c>
       <c r="C255" s="62" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D255" s="61" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="E255" s="63" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="F255" s="64"/>
       <c r="G255" s="64"/>
@@ -15483,13 +15488,13 @@
         <v>49</v>
       </c>
       <c r="C256" s="62" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D256" s="61" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="E256" s="63" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="F256" s="64"/>
       <c r="G256" s="64"/>
@@ -15524,13 +15529,13 @@
         <v>49</v>
       </c>
       <c r="C257" s="62" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D257" s="61" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="E257" s="63" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="F257" s="64"/>
       <c r="G257" s="64"/>
@@ -15565,13 +15570,13 @@
         <v>49</v>
       </c>
       <c r="C258" s="62" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D258" s="61" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="E258" s="63" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F258" s="64"/>
       <c r="G258" s="64"/>
@@ -15606,13 +15611,13 @@
         <v>49</v>
       </c>
       <c r="C259" s="62" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D259" s="61" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="E259" s="63" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="F259" s="64"/>
       <c r="G259" s="64"/>
@@ -15647,13 +15652,13 @@
         <v>49</v>
       </c>
       <c r="C260" s="62" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D260" s="61" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="E260" s="63" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="F260" s="64"/>
       <c r="G260" s="64"/>
@@ -15688,13 +15693,13 @@
         <v>49</v>
       </c>
       <c r="C261" s="62" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D261" s="61" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="E261" s="63" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="F261" s="64"/>
       <c r="G261" s="64"/>
@@ -15729,13 +15734,13 @@
         <v>49</v>
       </c>
       <c r="C262" s="62" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D262" s="61" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="E262" s="63" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="F262" s="64"/>
       <c r="G262" s="64"/>
@@ -15770,13 +15775,13 @@
         <v>49</v>
       </c>
       <c r="C263" s="62" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D263" s="61" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="E263" s="63" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="F263" s="64"/>
       <c r="G263" s="64"/>
@@ -15811,10 +15816,10 @@
         <v>49</v>
       </c>
       <c r="C264" s="62" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D264" s="61" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="E264" s="63" t="s">
         <v>80</v>
@@ -15852,10 +15857,10 @@
         <v>49</v>
       </c>
       <c r="C265" s="62" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D265" s="61" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="E265" s="63" t="s">
         <v>90</v>
@@ -15895,13 +15900,13 @@
         <v>49</v>
       </c>
       <c r="C266" s="62" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D266" s="61" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="E266" s="63" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="F266" s="64"/>
       <c r="G266" s="64"/>
@@ -15936,13 +15941,13 @@
         <v>49</v>
       </c>
       <c r="C267" s="62" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D267" s="61" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="E267" s="63" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="F267" s="64"/>
       <c r="G267" s="64"/>
@@ -15977,13 +15982,13 @@
         <v>49</v>
       </c>
       <c r="C268" s="62" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D268" s="61" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E268" s="63" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="F268" s="64"/>
       <c r="G268" s="64"/>
@@ -16018,13 +16023,13 @@
         <v>49</v>
       </c>
       <c r="C269" s="62" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D269" s="61" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="E269" s="63" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="F269" s="64"/>
       <c r="G269" s="64"/>
@@ -16059,13 +16064,13 @@
         <v>49</v>
       </c>
       <c r="C270" s="62" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D270" s="61" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="E270" s="63" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="F270" s="64"/>
       <c r="G270" s="64"/>
@@ -16100,13 +16105,13 @@
         <v>49</v>
       </c>
       <c r="C271" s="62" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D271" s="61" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="E271" s="63" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="F271" s="64"/>
       <c r="G271" s="64"/>
@@ -16141,13 +16146,13 @@
         <v>49</v>
       </c>
       <c r="C272" s="62" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D272" s="61" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="E272" s="63" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="F272" s="64"/>
       <c r="G272" s="64"/>
@@ -16182,13 +16187,13 @@
         <v>49</v>
       </c>
       <c r="C273" s="62" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D273" s="61" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="E273" s="63" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="F273" s="64"/>
       <c r="G273" s="64"/>
@@ -16223,13 +16228,13 @@
         <v>49</v>
       </c>
       <c r="C274" s="62" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D274" s="61" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="E274" s="63" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="F274" s="64"/>
       <c r="G274" s="64"/>
@@ -16264,13 +16269,13 @@
         <v>49</v>
       </c>
       <c r="C275" s="62" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D275" s="61" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="E275" s="63" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="F275" s="64"/>
       <c r="G275" s="64"/>
@@ -16305,13 +16310,13 @@
         <v>49</v>
       </c>
       <c r="C276" s="62" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D276" s="61" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="E276" s="63" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="F276" s="64"/>
       <c r="G276" s="64"/>
@@ -16346,13 +16351,13 @@
         <v>49</v>
       </c>
       <c r="C277" s="62" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D277" s="61" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="E277" s="63" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="F277" s="64"/>
       <c r="G277" s="64"/>
@@ -16387,13 +16392,13 @@
         <v>49</v>
       </c>
       <c r="C278" s="62" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D278" s="61" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="E278" s="63" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="F278" s="64"/>
       <c r="G278" s="64"/>
@@ -16428,13 +16433,13 @@
         <v>49</v>
       </c>
       <c r="C279" s="62" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D279" s="61" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="E279" s="63" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="F279" s="64"/>
       <c r="G279" s="64"/>
@@ -16469,13 +16474,13 @@
         <v>49</v>
       </c>
       <c r="C280" s="62" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D280" s="61" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="E280" s="63" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="F280" s="64"/>
       <c r="G280" s="64"/>
@@ -16510,13 +16515,13 @@
         <v>49</v>
       </c>
       <c r="C281" s="62" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D281" s="61" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="E281" s="63" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="F281" s="64"/>
       <c r="G281" s="64"/>
@@ -16551,13 +16556,13 @@
         <v>49</v>
       </c>
       <c r="C282" s="62" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D282" s="61" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="E282" s="63" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="F282" s="64"/>
       <c r="G282" s="64"/>
@@ -16592,13 +16597,13 @@
         <v>49</v>
       </c>
       <c r="C283" s="62" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D283" s="61" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="E283" s="63" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="F283" s="64"/>
       <c r="G283" s="64"/>
@@ -16633,10 +16638,10 @@
         <v>49</v>
       </c>
       <c r="C284" s="62" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D284" s="61" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="E284" s="63" t="s">
         <v>80</v>
@@ -16674,10 +16679,10 @@
         <v>49</v>
       </c>
       <c r="C285" s="62" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D285" s="61" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E285" s="63" t="s">
         <v>90</v>
@@ -19421,42 +19426,42 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
     </row>
   </sheetData>
@@ -19494,22 +19499,22 @@
   <sheetData>
     <row r="1" spans="1:7" customHeight="1" ht="14.25">
       <c r="A1" s="26" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B1" s="11" t="s">
         <v>27</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="D1" s="72" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="G1" s="39" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
     </row>
     <row r="2" spans="1:7" customHeight="1" ht="14.25">
@@ -19517,13 +19522,13 @@
         <v>50</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C2" s="70" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="D2" s="73" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
     </row>
     <row r="3" spans="1:7" customHeight="1" ht="14.25">
@@ -19531,13 +19536,13 @@
         <v>59</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C3" s="70" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="D3" s="74" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
     </row>
     <row r="4" spans="1:7" customHeight="1" ht="14.25">
@@ -19545,13 +19550,13 @@
         <v>63</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C4" s="70" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="D4" s="75" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="5" spans="1:7" customHeight="1" ht="14.25">
@@ -19559,13 +19564,13 @@
         <v>73</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C5" s="70" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="D5" s="74" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
     </row>
     <row r="6" spans="1:7" customHeight="1" ht="14.25">
@@ -19573,13 +19578,13 @@
         <v>75</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C6" s="70" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="D6" s="75" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
     </row>
     <row r="7" spans="1:7" customHeight="1" ht="14.5">
@@ -19587,13 +19592,13 @@
         <v>77</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C7" s="70" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="D7" s="75" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
     </row>
     <row r="8" spans="1:7" customHeight="1" ht="14.5">
@@ -19601,13 +19606,13 @@
         <v>65</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C8" s="70" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="D8" s="75" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
     </row>
     <row r="9" spans="1:7" customHeight="1" ht="14.5">
@@ -19615,125 +19620,125 @@
         <v>61</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C9" s="70" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="D9" s="75" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
     </row>
     <row r="10" spans="1:7" customHeight="1" ht="43.5">
       <c r="A10" s="5" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C10" s="71" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="D10" s="74" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="11" spans="1:7" customHeight="1" ht="14.25">
       <c r="A11" s="5" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C11" s="70" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="D11" s="75" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
     </row>
     <row r="12" spans="1:7" customHeight="1" ht="14.25">
       <c r="A12" s="5" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C12" s="70" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="D12" s="75" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
     </row>
     <row r="13" spans="1:7" customHeight="1" ht="14.25">
       <c r="A13" s="5" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C13" s="70" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="D13" s="75" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
     </row>
     <row r="14" spans="1:7" customHeight="1" ht="14.25">
       <c r="A14" s="5" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C14" s="70" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="D14" s="75" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
     </row>
     <row r="15" spans="1:7" customHeight="1" ht="14.25">
       <c r="A15" s="5" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C15" s="70">
         <v>521</v>
       </c>
       <c r="D15" s="75" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
     </row>
     <row r="16" spans="1:7" customHeight="1" ht="14.25">
       <c r="A16" s="77" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C16" s="79" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="D16" s="75" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
     </row>
     <row r="17" spans="1:7" customHeight="1" ht="14.25">
       <c r="A17" s="78" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="B17" s="76" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C17" s="80" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="D17" s="75" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
     </row>
     <row r="18" spans="1:7" customHeight="1" ht="14.25"/>
@@ -20722,7 +20727,7 @@
     </row>
     <row r="2" spans="1:6" customHeight="1" ht="14.25">
       <c r="A2" s="4" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>70</v>
@@ -20730,7 +20735,7 @@
     </row>
     <row r="3" spans="1:6" customHeight="1" ht="14.25">
       <c r="A3" s="4" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>53</v>

</xml_diff>